<commit_message>
feat: Nang cap toan bo he thong AutoBillApp (VAT 2 chieu, Run-Span Word, toi uu Excel, giao dien van phong, don dep repo)
</commit_message>
<xml_diff>
--- a/templates/ĐỀ XUẤT VẬT TƯ.xlsx
+++ b/templates/ĐỀ XUẤT VẬT TƯ.xlsx
@@ -1426,16 +1426,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1377202</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>3985895</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>71717</xdr:rowOff>
+      <xdr:rowOff>71120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>136150</xdr:colOff>
+      <xdr:colOff>135890</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>157442</xdr:rowOff>
+      <xdr:rowOff>151765</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1446,8 +1446,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6686550" y="71120"/>
-          <a:ext cx="3940810" cy="474345"/>
+          <a:off x="4387215" y="71120"/>
+          <a:ext cx="6240145" cy="469265"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1466,9 +1466,7 @@
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
-        <a:bodyPr rot="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" anchorCtr="0" upright="1">
-          <a:noAutofit/>
-        </a:bodyPr>
+        <a:bodyPr rot="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" anchorCtr="0" upright="1"/>
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="ctr">

</xml_diff>

<commit_message>
fix & perf: toi uu hieu nang form chong mo man hinh, tang toc xuat zip 8x, giu nguyen gia bao gia va bo sung form nhap chung tu
</commit_message>
<xml_diff>
--- a/templates/ĐỀ XUẤT VẬT TƯ.xlsx
+++ b/templates/ĐỀ XUẤT VẬT TƯ.xlsx
@@ -7,8 +7,8 @@
     <workbookView windowWidth="23040" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Báo giá" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Báo giá" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="62">
   <si>
     <t>CN CÔNG TY TNHH MM MEGA MARKET VIỆT NAM TẠI TỈNH BÌNH ĐỊNH</t>
   </si>
@@ -151,6 +151,9 @@
     <t>{muc_dich}</t>
   </si>
   <si>
+    <t>{ton_kho}</t>
+  </si>
+  <si>
     <t>{nha_cung_cap}</t>
   </si>
   <si>
@@ -158,6 +161,9 @@
   </si>
   <si>
     <t>{so_luong}</t>
+  </si>
+  <si>
+    <t>{gia_niem_yet}</t>
   </si>
   <si>
     <t>{don_gia}</t>
@@ -304,14 +310,14 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <i/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="14"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
@@ -777,19 +783,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -805,6 +798,19 @@
       <right style="thin">
         <color auto="1"/>
       </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -914,148 +920,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="23" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="8" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="23" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="23" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="14">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="4" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1068,10 +1074,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1106,6 +1111,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1115,49 +1122,33 @@
     <xf numFmtId="178" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="3"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="3"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1170,7 +1161,7 @@
     <xf numFmtId="1" fontId="14" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="179" fontId="14" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="14" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="179" fontId="14" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1181,7 +1172,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="18" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="179" fontId="19" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="19" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1196,7 +1187,6 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1301,13 +1291,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip r:embed="rId1"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
@@ -1324,26 +1308,8 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1369,13 +1335,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip r:embed="rId1"/>
         <a:srcRect/>
         <a:stretch>
           <a:fillRect/>
@@ -1392,26 +1352,8 @@
         <a:noFill/>
         <a:ln>
           <a:noFill/>
+          <a:prstDash val="solid"/>
         </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1421,187 +1363,6 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3985895</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>71120</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>135890</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>151765</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Text Box 16"/>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4387215" y="71120"/>
-          <a:ext cx="6240145" cy="469265"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FFFFFF"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:schemeClr val="bg1">
-              <a:lumMod val="100000"/>
-              <a:lumOff val="0"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr rot="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" anchorCtr="0" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:lnSpc>
-              <a:spcPct val="150000"/>
-            </a:lnSpc>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1">
-              <a:effectLst/>
-              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            </a:rPr>
-            <a:t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:effectLst/>
-            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:lnSpc>
-              <a:spcPct val="150000"/>
-            </a:lnSpc>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" u="sng">
-              <a:effectLst/>
-              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            </a:rPr>
-            <a:t>Độc lập – Tự do – Hạnh phúc</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:effectLst/>
-            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400">
-              <a:effectLst/>
-              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:effectLst/>
-            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1247775</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Text Box 1"/>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="12898755" y="0"/>
-          <a:ext cx="2283460" cy="289560"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FFFFFF"/>
-        </a:solidFill>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:miter lim="800000"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr rot="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="t" anchorCtr="0" upright="1">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr">
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:effectLst/>
-              <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-              <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            </a:rPr>
-            <a:t>BM-TCKT-MS-01R1</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:effectLst/>
-            <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-            <a:ea typeface="Times New Roman" panose="02020603050405020304" pitchFamily="12"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -1623,13 +1384,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1642,6 +1397,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1939,209 +1697,198 @@
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="9.13888888888889" style="38"/>
+    <col min="1" max="1" width="9.13888888888889" style="33" customWidth="1"/>
     <col min="2" max="2" width="11.1388888888889" customWidth="1"/>
     <col min="3" max="3" width="64.5740740740741" customWidth="1"/>
-    <col min="4" max="4" width="21.8518518518519" style="39" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.8518518518519" style="34" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="21.8518518518519" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="40"/>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
+      <c r="A1" s="35"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="42"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43" t="s">
+      <c r="A2" s="37"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="42"/>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43" t="s">
+      <c r="A3" s="37"/>
+      <c r="B3" s="38"/>
+      <c r="C3" s="38" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="40"/>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-    </row>
-    <row r="5" ht="25.8" spans="1:6">
-      <c r="A5" s="44" t="s">
+      <c r="A4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+    </row>
+    <row r="5" ht="25.8" customHeight="1" spans="1:6">
+      <c r="A5" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-    </row>
-    <row r="6" ht="25.8" spans="1:6">
-      <c r="A6" s="42" t="s">
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+    </row>
+    <row r="6" ht="25.8" customHeight="1" spans="1:6">
+      <c r="A6" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="42" t="s">
+      <c r="A7" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="47" t="s">
+      <c r="A9" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="50" t="s">
+      <c r="E9" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="48" t="s">
+      <c r="F9" s="43" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A10" s="51">
+      <c r="A10" s="46">
         <v>1</v>
       </c>
-      <c r="B10" s="52">
+      <c r="B10" s="47">
         <v>213675</v>
       </c>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="54"/>
-      <c r="E10" s="55">
+      <c r="D10" s="49"/>
+      <c r="E10" s="50">
         <v>78466</v>
       </c>
-      <c r="F10" s="56">
+      <c r="F10" s="51">
         <v>0.08</v>
       </c>
     </row>
     <row r="11" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A11" s="51">
+      <c r="A11" s="46">
         <v>2</v>
       </c>
-      <c r="B11" s="57">
+      <c r="B11" s="52">
         <v>72583</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="54"/>
-      <c r="E11" s="55">
+      <c r="D11" s="49"/>
+      <c r="E11" s="50">
         <v>62584</v>
       </c>
-      <c r="F11" s="56">
+      <c r="F11" s="51">
         <v>0.08</v>
       </c>
     </row>
     <row r="12" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A12" s="51">
+      <c r="A12" s="46">
         <v>3</v>
       </c>
-      <c r="B12" s="52">
+      <c r="B12" s="47">
         <v>253915</v>
       </c>
-      <c r="C12" s="59" t="s">
+      <c r="C12" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="54"/>
-      <c r="E12" s="55">
+      <c r="D12" s="49"/>
+      <c r="E12" s="50">
         <v>36670</v>
       </c>
-      <c r="F12" s="56">
+      <c r="F12" s="51">
         <v>0.08</v>
       </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A13" s="51">
+      <c r="A13" s="46">
         <v>4</v>
       </c>
-      <c r="B13" s="52">
+      <c r="B13" s="47">
         <v>139972</v>
       </c>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="54"/>
-      <c r="E13" s="55">
+      <c r="D13" s="49"/>
+      <c r="E13" s="50">
         <v>274649</v>
       </c>
-      <c r="F13" s="56">
+      <c r="F13" s="51">
         <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="D14" s="60"/>
-      <c r="E14" s="61"/>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="62" t="s">
+      <c r="E14" s="55"/>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="56" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="43" t="s">
+      <c r="B17" s="36"/>
+      <c r="C17" s="36"/>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="43"/>
-      <c r="D18"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="43" t="s">
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43"/>
-      <c r="D19"/>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="63" t="s">
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="63"/>
-      <c r="C20" s="63"/>
-      <c r="D20"/>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="43" t="s">
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="43"/>
-      <c r="D21"/>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="41"/>
-      <c r="B22" s="41"/>
-      <c r="C22" s="41"/>
-      <c r="D22"/>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23"/>
-      <c r="C23" s="64" t="s">
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="36"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="36"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="C23" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="D23"/>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24"/>
-      <c r="C24" s="64" t="s">
+    </row>
+    <row r="24" spans="1:3">
+      <c r="C24" s="58" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2185,151 +1932,134 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="9.13888888888889" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="5.85185185185185" style="2" customWidth="1"/>
     <col min="2" max="2" width="71.5740740740741" style="2" customWidth="1"/>
     <col min="3" max="3" width="24.8518518518519" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.13888888888889" style="2"/>
+    <col min="4" max="4" width="9.13888888888889" style="2" customWidth="1"/>
     <col min="5" max="5" width="26.1388888888889" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.4259259259259" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.5740740740741" style="2" customWidth="1"/>
     <col min="8" max="8" width="20.7777777777778" style="2" customWidth="1"/>
     <col min="9" max="10" width="18.8518518518519" style="2" customWidth="1"/>
-    <col min="11" max="11" width="14.1388888888889" style="2" customWidth="1"/>
+    <col min="11" max="11" width="16.462962962963" style="2" customWidth="1"/>
     <col min="12" max="12" width="14.712962962963" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="9.13888888888889" style="2"/>
+    <col min="13" max="16384" width="9.13888888888889" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.8" spans="1:14">
+    <row r="1" ht="16.8" customHeight="1" spans="1:12">
       <c r="A1" s="3"/>
     </row>
-    <row r="5" ht="20.4" spans="1:14">
+    <row r="5" ht="20.4" customHeight="1" spans="1:12">
       <c r="A5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
       <c r="K5" s="5"/>
     </row>
-    <row r="6" ht="15.6" spans="1:14">
+    <row r="6" ht="15.6" customHeight="1" spans="1:12">
       <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="7"/>
-    </row>
-    <row r="7" ht="17.4" spans="1:14">
-      <c r="A7" s="8"/>
-      <c r="E7" s="8"/>
-    </row>
-    <row r="8" ht="17.4" spans="1:14">
-      <c r="A8" s="9"/>
+    </row>
+    <row r="7" ht="17.4" customHeight="1" spans="1:12">
+      <c r="A7" s="7"/>
+      <c r="E7" s="7"/>
+    </row>
+    <row r="8" ht="17.4" customHeight="1" spans="1:12">
+      <c r="A8" s="8"/>
       <c r="B8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="9" ht="17.4" spans="1:14">
-      <c r="A9" s="9"/>
+    <row r="9" ht="17.4" customHeight="1" spans="1:12">
+      <c r="A9" s="8"/>
       <c r="B9" s="5"/>
-      <c r="E9" s="9"/>
-      <c r="H9" s="9"/>
-    </row>
-    <row r="10" ht="47.25" customHeight="1" spans="1:14">
-      <c r="A10" s="10" t="s">
+      <c r="E9" s="8"/>
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" ht="47.25" customHeight="1" spans="1:12">
+      <c r="A10" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="J10" s="10" t="s">
+      <c r="J10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="K10" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="L10" s="12"/>
-      <c r="M10" s="7"/>
-    </row>
-    <row r="11" ht="21" customHeight="1" spans="1:14">
-      <c r="A11" s="13" t="s">
+      <c r="L10" s="11"/>
+    </row>
+    <row r="11" ht="21" customHeight="1" spans="1:12">
+      <c r="A11" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="13"/>
-      <c r="E11" s="15" t="s">
+      <c r="D11" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="E11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="16" t="s">
+      <c r="F11" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17" t="s">
+      <c r="G11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="17" t="s">
+      <c r="H11" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="K11" s="17" t="s">
+      <c r="I11" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="L11" s="18"/>
-      <c r="M11" s="7"/>
-    </row>
-    <row r="12" ht="19.5" customHeight="1" spans="1:14">
-      <c r="A12" s="19" t="s">
+      <c r="J11" s="16" t="s">
         <v>46</v>
+      </c>
+      <c r="K11" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="L11" s="17"/>
+    </row>
+    <row r="12" ht="19.5" customHeight="1" spans="1:12">
+      <c r="A12" s="18" t="s">
+        <v>48</v>
       </c>
       <c r="B12" s="19"/>
       <c r="C12" s="19"/>
@@ -2338,180 +2068,156 @@
       <c r="F12" s="19"/>
       <c r="G12" s="19"/>
       <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="20" t="s">
-        <v>47</v>
-      </c>
-      <c r="K12" s="21"/>
-      <c r="L12" s="22"/>
-      <c r="N12" s="7"/>
-    </row>
-    <row r="13" ht="19.5" customHeight="1" spans="1:14">
-      <c r="A13" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="26" t="s">
+      <c r="I12" s="20"/>
+      <c r="J12" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="K13" s="21"/>
-      <c r="L13" s="22"/>
-      <c r="N13" s="7"/>
-    </row>
-    <row r="14" ht="19.5" customHeight="1" spans="1:14">
-      <c r="A14" s="27" t="s">
+      <c r="K12" s="22"/>
+      <c r="L12" s="23"/>
+    </row>
+    <row r="13" ht="19.5" customHeight="1" spans="1:12">
+      <c r="A13" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="26" t="s">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="K14" s="21"/>
-      <c r="L14" s="22"/>
-      <c r="N14" s="7"/>
-    </row>
-    <row r="15" ht="19.5" customHeight="1" spans="1:14">
-      <c r="A15" s="30"/>
-      <c r="J15" s="31"/>
+      <c r="K13" s="22"/>
+      <c r="L13" s="23"/>
+    </row>
+    <row r="14" ht="19.5" customHeight="1" spans="1:12">
+      <c r="A14" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="K14" s="22"/>
+      <c r="L14" s="23"/>
+    </row>
+    <row r="15" ht="19.5" customHeight="1" spans="1:12">
+      <c r="A15" s="26"/>
+      <c r="J15" s="1"/>
       <c r="K15" s="1"/>
-      <c r="L15" s="22"/>
-      <c r="N15" s="7"/>
-    </row>
-    <row r="16" ht="19.5" customHeight="1" spans="1:14">
-      <c r="I16" s="32" t="s">
-        <v>52</v>
+      <c r="L15" s="23"/>
+    </row>
+    <row r="16" ht="19.5" customHeight="1" spans="1:12">
+      <c r="I16" s="27" t="s">
+        <v>54</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="N16" s="7"/>
-    </row>
-    <row r="17" ht="19.5" customHeight="1" spans="1:14">
-      <c r="I17" s="33"/>
-      <c r="N17" s="7"/>
-    </row>
-    <row r="18" ht="17.4" spans="1:14">
-      <c r="A18" s="34" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="34"/>
-      <c r="C18" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34" t="s">
+    </row>
+    <row r="17" ht="19.5" customHeight="1" spans="1:12">
+      <c r="I17" s="28"/>
+    </row>
+    <row r="18" ht="17.4" customHeight="1" spans="1:12">
+      <c r="A18" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34" t="s">
+      <c r="C18" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="M18" s="7"/>
-    </row>
-    <row r="19" ht="18" spans="1:14">
-      <c r="A19" s="35"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="36"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="M19" s="7"/>
-    </row>
-    <row r="20" ht="20.25" customHeight="1" spans="1:14">
-      <c r="A20" s="35"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="36"/>
-      <c r="K20" s="36"/>
-      <c r="M20" s="7"/>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="23.25" customHeight="1" spans="1:14">
-      <c r="A21" s="35"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="36"/>
-      <c r="J21" s="36"/>
-      <c r="K21" s="36"/>
+      <c r="F18" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" s="29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" spans="1:12">
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+    </row>
+    <row r="20" ht="20.25" customHeight="1" spans="1:12">
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="23.25" customHeight="1" spans="1:12">
+      <c r="A21" s="30"/>
+      <c r="B21" s="30"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="G21" s="29"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
       <c r="L21" s="2"/>
-      <c r="M21" s="31"/>
-    </row>
-    <row r="22" s="1" customFormat="1" ht="18" spans="1:14">
-      <c r="A22" s="35"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="18" customHeight="1" spans="1:12">
+      <c r="A22" s="30"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" ht="18" spans="1:14">
-      <c r="A23" s="35"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="36"/>
-      <c r="J23" s="36"/>
-      <c r="K23" s="36"/>
-    </row>
-    <row r="24" ht="17.4" spans="1:14">
-      <c r="A24" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37" t="s">
+    <row r="23" ht="18" customHeight="1" spans="1:12">
+      <c r="A23" s="30"/>
+      <c r="B23" s="30"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+    </row>
+    <row r="24" ht="17.4" customHeight="1" spans="1:12">
+      <c r="A24" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="J24" s="37"/>
-      <c r="K24" s="37"/>
+      <c r="C24" s="32"/>
+      <c r="F24" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="I24" s="32" t="s">
+        <v>61</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
refactor: redesign manual entry mode layout, fix tax rate display bug, improve unit price calculation for quotes, allow unicode in zip filenames
</commit_message>
<xml_diff>
--- a/templates/ĐỀ XUẤT VẬT TƯ.xlsx
+++ b/templates/ĐỀ XUẤT VẬT TƯ.xlsx
@@ -193,7 +193,7 @@
     <t>{tong_cong}</t>
   </si>
   <si>
-    <t>{ngay_thang_nam}</t>
+    <t>Gia Lai, ngày {ngay_ky} tháng {thang_ky} năm {nam_ky}</t>
   </si>
   <si>
     <t>Người đề xuất</t>
@@ -1061,7 +1061,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1128,11 +1128,12 @@
     <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="3"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="3"/>
@@ -1697,198 +1698,198 @@
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="9.13888888888889" style="33" customWidth="1"/>
+    <col min="1" max="1" width="9.13888888888889" style="34" customWidth="1"/>
     <col min="2" max="2" width="11.1388888888889" customWidth="1"/>
     <col min="3" max="3" width="64.5740740740741" customWidth="1"/>
-    <col min="4" max="4" width="21.8518518518519" style="34" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.8518518518519" style="35" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="21.8518518518519" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="35"/>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
+      <c r="A1" s="36"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="37"/>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38" t="s">
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="37"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38" t="s">
+      <c r="A3" s="38"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="35"/>
-      <c r="B4" s="36"/>
-      <c r="C4" s="36"/>
+      <c r="A4" s="36"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="37"/>
     </row>
     <row r="5" ht="25.8" customHeight="1" spans="1:6">
-      <c r="A5" s="39" t="s">
+      <c r="A5" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
     </row>
     <row r="6" ht="25.8" customHeight="1" spans="1:6">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="38"/>
-      <c r="C7" s="38"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="42" t="s">
+      <c r="A9" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="43" t="s">
+      <c r="B9" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="43" t="s">
+      <c r="C9" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="44" t="s">
+      <c r="D9" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="45" t="s">
+      <c r="E9" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="43" t="s">
+      <c r="F9" s="44" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="10" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A10" s="46">
+      <c r="A10" s="47">
         <v>1</v>
       </c>
-      <c r="B10" s="47">
+      <c r="B10" s="48">
         <v>213675</v>
       </c>
-      <c r="C10" s="48" t="s">
+      <c r="C10" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="49"/>
-      <c r="E10" s="50">
+      <c r="D10" s="50"/>
+      <c r="E10" s="51">
         <v>78466</v>
       </c>
-      <c r="F10" s="51">
+      <c r="F10" s="52">
         <v>0.08</v>
       </c>
     </row>
     <row r="11" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A11" s="46">
+      <c r="A11" s="47">
         <v>2</v>
       </c>
-      <c r="B11" s="52">
+      <c r="B11" s="53">
         <v>72583</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="49"/>
-      <c r="E11" s="50">
+      <c r="D11" s="50"/>
+      <c r="E11" s="51">
         <v>62584</v>
       </c>
-      <c r="F11" s="51">
+      <c r="F11" s="52">
         <v>0.08</v>
       </c>
     </row>
     <row r="12" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A12" s="46">
+      <c r="A12" s="47">
         <v>3</v>
       </c>
-      <c r="B12" s="47">
+      <c r="B12" s="48">
         <v>253915</v>
       </c>
-      <c r="C12" s="54" t="s">
+      <c r="C12" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="D12" s="49"/>
-      <c r="E12" s="50">
+      <c r="D12" s="50"/>
+      <c r="E12" s="51">
         <v>36670</v>
       </c>
-      <c r="F12" s="51">
+      <c r="F12" s="52">
         <v>0.08</v>
       </c>
     </row>
     <row r="13" ht="25.5" customHeight="1" spans="1:6">
-      <c r="A13" s="46">
+      <c r="A13" s="47">
         <v>4</v>
       </c>
-      <c r="B13" s="47">
+      <c r="B13" s="48">
         <v>139972</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="49"/>
-      <c r="E13" s="50">
+      <c r="D13" s="50"/>
+      <c r="E13" s="51">
         <v>274649</v>
       </c>
-      <c r="F13" s="51">
+      <c r="F13" s="52">
         <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="E14" s="55"/>
+      <c r="E14" s="56"/>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" s="56" t="s">
+      <c r="A17" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="38" t="s">
+      <c r="A19" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" s="57" t="s">
+      <c r="A20" s="58" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
+      <c r="B21" s="39"/>
+      <c r="C21" s="39"/>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" s="36"/>
-      <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
     </row>
     <row r="23" spans="1:3">
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="59" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="59" t="s">
         <v>20</v>
       </c>
     </row>
@@ -2108,124 +2109,126 @@
       <c r="J14" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="K14" s="22"/>
-      <c r="L14" s="23"/>
+      <c r="K14" s="26"/>
+      <c r="L14" s="26"/>
     </row>
     <row r="15" ht="19.5" customHeight="1" spans="1:12">
-      <c r="A15" s="26"/>
+      <c r="A15" s="27"/>
       <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="23"/>
     </row>
     <row r="16" ht="19.5" customHeight="1" spans="1:12">
-      <c r="I16" s="27" t="s">
+      <c r="H16" s="28" t="s">
         <v>54</v>
       </c>
-      <c r="L16" s="1"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="28"/>
+      <c r="L16" s="28"/>
     </row>
     <row r="17" ht="19.5" customHeight="1" spans="1:12">
-      <c r="I17" s="28"/>
+      <c r="I17" s="29"/>
     </row>
     <row r="18" ht="17.4" customHeight="1" spans="1:12">
-      <c r="A18" s="29" t="s">
+      <c r="A18" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="C18" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="29" t="s">
+      <c r="F18" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="I18" s="29" t="s">
+      <c r="I18" s="30" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" spans="1:12">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="29"/>
-      <c r="G19" s="29"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="31"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
+      <c r="A19" s="31"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
     </row>
     <row r="20" ht="20.25" customHeight="1" spans="1:12">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="29"/>
-      <c r="G20" s="29"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
+      <c r="A20" s="31"/>
+      <c r="B20" s="31"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
     </row>
     <row r="21" s="1" customFormat="1" ht="23.25" customHeight="1" spans="1:12">
-      <c r="A21" s="30"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="31"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
+      <c r="A21" s="31"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
       <c r="L21" s="2"/>
     </row>
     <row r="22" s="1" customFormat="1" ht="18" customHeight="1" spans="1:12">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="31"/>
-      <c r="I22" s="31"/>
-      <c r="J22" s="31"/>
-      <c r="K22" s="31"/>
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="32"/>
+      <c r="I22" s="32"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
       <c r="L22" s="2"/>
     </row>
     <row r="23" ht="18" customHeight="1" spans="1:12">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="31"/>
-      <c r="J23" s="31"/>
-      <c r="K23" s="31"/>
+      <c r="A23" s="31"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="30"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="32"/>
+      <c r="K23" s="32"/>
     </row>
     <row r="24" ht="17.4" customHeight="1" spans="1:12">
       <c r="A24" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="F24" s="32" t="s">
+      <c r="C24" s="33"/>
+      <c r="F24" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="I24" s="32" t="s">
+      <c r="I24" s="33" t="s">
         <v>61</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A6:J6"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="A13:I13"/>
     <mergeCell ref="A14:I14"/>
+    <mergeCell ref="H16:L16"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="F18:H18"/>

</xml_diff>